<commit_message>
consistently use "class" instead of "employee_class" as column names in the stacked tables
All tests passed
</commit_message>
<xml_diff>
--- a/refactor/source_data/FRS_rules_table.xlsx
+++ b/refactor/source_data/FRS_rules_table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gang Chen\OneDrive - University at Albany - SUNY\r-projects\Florida-FRS-main_generalizable\refactor\source_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livealbany-my.sharepoint.com/personal/gchen3_albany_edu/Documents/R-projects/Florida-FRS-main_generalizable/refactor/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFD9A63-AB49-43A6-9E65-911658A94A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{1CFD9A63-AB49-43A6-9E65-911658A94A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F99790BC-756A-44D2-8A29-E7C9DA2EA3C7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0527D138-38C7-42E4-8E45-E7785205E030}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0527D138-38C7-42E4-8E45-E7785205E030}"/>
   </bookViews>
   <sheets>
     <sheet name="benmult" sheetId="1" r:id="rId1"/>
@@ -144,12 +144,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="32">
   <si>
     <t>system</t>
-  </si>
-  <si>
-    <t>class_name</t>
   </si>
   <si>
     <t>tier_group</t>
@@ -374,7 +371,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -415,9 +412,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -922,42 +916,42 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="J2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D3" s="6">
         <v>0</v>
@@ -983,13 +977,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D4" s="6">
         <v>0</v>
@@ -1015,13 +1009,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D5" s="6">
         <v>0</v>
@@ -1047,13 +1041,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
@@ -1091,13 +1085,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D8" s="6">
         <v>65</v>
@@ -1123,13 +1117,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D9" s="6">
         <v>64</v>
@@ -1155,13 +1149,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D10" s="6">
         <v>63</v>
@@ -1187,13 +1181,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="17" t="s">
         <v>4</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>5</v>
       </c>
       <c r="D11" s="6">
         <v>62</v>
@@ -1231,13 +1225,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>4</v>
-      </c>
       <c r="C13" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D13" s="6">
         <v>0</v>
@@ -1263,13 +1257,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C15" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -1295,13 +1289,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C16" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16" s="9">
         <v>0</v>
@@ -1327,13 +1321,13 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C17" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" s="9">
         <v>0</v>
@@ -1359,13 +1353,13 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C18" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D18" s="9">
         <v>0</v>
@@ -1403,13 +1397,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C20" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" s="9">
         <v>68</v>
@@ -1435,13 +1429,13 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C21" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D21" s="9">
         <v>67</v>
@@ -1467,13 +1461,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C22" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22" s="9">
         <v>66</v>
@@ -1499,13 +1493,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C23" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D23" s="9">
         <v>65</v>
@@ -1543,13 +1537,13 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>4</v>
-      </c>
       <c r="C25" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D25" s="9">
         <v>0</v>
@@ -1583,13 +1577,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C27" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D27" s="12">
         <v>0</v>
@@ -1615,13 +1609,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C28" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D28" s="12">
         <v>0</v>
@@ -1647,13 +1641,13 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C29" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" s="12">
         <v>0</v>
@@ -1679,13 +1673,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B30" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C30" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D30" s="12">
         <v>0</v>
@@ -1723,13 +1717,13 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C32" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D32" s="12">
         <v>68</v>
@@ -1755,13 +1749,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C33" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" s="12">
         <v>67</v>
@@ -1787,13 +1781,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C34" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D34" s="12">
         <v>66</v>
@@ -1819,13 +1813,13 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B35" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C35" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D35" s="12">
         <v>65</v>
@@ -1863,13 +1857,13 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="11" t="s">
-        <v>4</v>
-      </c>
       <c r="C37" s="19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D37" s="12">
         <v>0</v>
@@ -1911,13 +1905,13 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D40" s="15">
         <v>0</v>
@@ -1943,13 +1937,13 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D41" s="15">
         <v>0</v>
@@ -1975,13 +1969,13 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D42" s="15">
         <v>0</v>
@@ -2007,13 +2001,13 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D43" s="15">
         <v>0</v>
@@ -2051,13 +2045,13 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D45" s="15">
         <v>58</v>
@@ -2083,13 +2077,13 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D46" s="15">
         <v>57</v>
@@ -2115,13 +2109,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D47" s="15">
         <v>56</v>
@@ -2147,13 +2141,13 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48" s="15">
         <v>55</v>
@@ -2191,13 +2185,13 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D50" s="15">
         <v>0</v>
@@ -2223,13 +2217,13 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D52" s="15">
         <v>0</v>
@@ -2255,13 +2249,13 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D53" s="15">
         <v>0</v>
@@ -2287,13 +2281,13 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D54" s="15">
         <v>0</v>
@@ -2319,13 +2313,13 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D55" s="15">
         <v>0</v>
@@ -2363,13 +2357,13 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D57" s="15">
         <v>63</v>
@@ -2395,13 +2389,13 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D58" s="15">
         <v>62</v>
@@ -2427,13 +2421,13 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D59" s="15">
         <v>61</v>
@@ -2459,13 +2453,13 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D60" s="15">
         <v>60</v>
@@ -2503,13 +2497,13 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B62" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C62" s="20" t="s">
         <v>16</v>
-      </c>
-      <c r="C62" s="20" t="s">
-        <v>17</v>
       </c>
       <c r="D62" s="15">
         <v>0</v>
@@ -2595,13 +2589,13 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D69" s="15">
         <v>63</v>
@@ -2627,13 +2621,13 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B70" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" s="15">
         <v>62</v>
@@ -2659,13 +2653,13 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C71" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D71" s="15">
         <v>61</v>
@@ -2691,13 +2685,13 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C72" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D72" s="15">
         <v>60</v>
@@ -2735,13 +2729,13 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C74" s="20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D74" s="15">
         <v>0</v>
@@ -2767,13 +2761,13 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B77" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C77" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D77" s="25">
         <v>0</v>
@@ -2799,13 +2793,13 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B78" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C78" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D78" s="25">
         <v>0</v>
@@ -2831,13 +2825,13 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B79" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C79" s="24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D79" s="25">
         <v>0</v>
@@ -2863,13 +2857,13 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B80" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C80" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D80" s="25">
         <v>0</v>
@@ -2895,13 +2889,13 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B81" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C81" s="24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D81" s="25">
         <v>0</v>
@@ -2927,13 +2921,13 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B82" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C82" s="24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D82" s="25">
         <v>0</v>
@@ -2971,13 +2965,13 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B84" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C84" s="24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D84" s="25">
         <v>0</v>
@@ -3003,13 +2997,13 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B85" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C85" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D85" s="25">
         <v>0</v>
@@ -3035,13 +3029,13 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B86" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C86" s="24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D86" s="25">
         <v>0</v>
@@ -3067,13 +3061,13 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B87" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C87" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D87" s="25">
         <v>0</v>
@@ -3099,13 +3093,13 @@
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B88" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C88" s="24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D88" s="25">
         <v>0</v>
@@ -3131,13 +3125,13 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="24" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B89" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C89" s="24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D89" s="25">
         <v>0</v>
@@ -3181,13 +3175,13 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D92" s="29">
         <v>0</v>
@@ -3213,13 +3207,13 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D93" s="29">
         <v>0</v>
@@ -3245,13 +3239,13 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D94" s="29">
         <v>0</v>
@@ -3277,13 +3271,13 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D95" s="29">
         <v>0</v>
@@ -3309,13 +3303,13 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D96" s="29">
         <v>0</v>
@@ -3341,13 +3335,13 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D97" s="29">
         <v>0</v>
@@ -3391,13 +3385,13 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B100" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C100" s="31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D100" s="32">
         <v>0</v>
@@ -3423,13 +3417,13 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B101" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C101" s="31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D101" s="32">
         <v>0</v>
@@ -3455,13 +3449,13 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B102" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C102" s="31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D102" s="32">
         <v>0</v>
@@ -3487,13 +3481,13 @@
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B103" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C103" s="31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D103" s="32">
         <v>0</v>
@@ -3519,13 +3513,13 @@
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B104" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C104" s="31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D104" s="32">
         <v>0</v>
@@ -3551,13 +3545,13 @@
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B105" s="31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C105" s="31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D105" s="32">
         <v>0</v>
@@ -3599,13 +3593,13 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B108" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C108" s="34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D108" s="35">
         <v>0</v>
@@ -3631,13 +3625,13 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B109" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C109" s="34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D109" s="35">
         <v>0</v>
@@ -3663,13 +3657,13 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B110" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C110" s="34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D110" s="35">
         <v>0</v>
@@ -3695,13 +3689,13 @@
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B111" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C111" s="34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D111" s="35">
         <v>0</v>
@@ -3727,13 +3721,13 @@
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B112" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C112" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D112" s="35">
         <v>0</v>
@@ -3759,13 +3753,13 @@
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B113" s="34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C113" s="34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D113" s="35">
         <v>0</v>
@@ -3807,13 +3801,13 @@
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B116" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C116" s="37" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D116" s="38">
         <v>0</v>
@@ -3839,13 +3833,13 @@
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B117" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C117" s="37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D117" s="38">
         <v>0</v>
@@ -3871,13 +3865,13 @@
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B118" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C118" s="37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D118" s="38">
         <v>0</v>
@@ -3903,13 +3897,13 @@
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B119" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C119" s="37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D119" s="38">
         <v>0</v>
@@ -3935,13 +3929,13 @@
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B120" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C120" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D120" s="38">
         <v>0</v>
@@ -3967,13 +3961,13 @@
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" s="37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B121" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C121" s="37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D121" s="38">
         <v>0</v>
@@ -4223,473 +4217,473 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="40" t="s">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
         <v>18</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="41" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="42" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="42" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="41" t="s">
-        <v>19</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="41" t="s">
-        <v>19</v>
+      <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="41" t="s">
-        <v>19</v>
+      <c r="A25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="42" t="s">
-        <v>4</v>
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>3</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="42" t="s">
-        <v>4</v>
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
+        <v>3</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="42" t="s">
-        <v>4</v>
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="42" t="s">
-        <v>16</v>
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>15</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="42" t="s">
-        <v>16</v>
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="42" t="s">
-        <v>16</v>
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="42" t="s">
-        <v>20</v>
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>19</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="42" t="s">
-        <v>20</v>
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="42" t="s">
-        <v>20</v>
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="42" t="s">
-        <v>21</v>
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>20</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="42" t="s">
-        <v>21</v>
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
       </c>
       <c r="C36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B37" s="42" t="s">
-        <v>21</v>
+      <c r="A37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" t="s">
+        <v>20</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" s="42" t="s">
-        <v>22</v>
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B39" s="42" t="s">
-        <v>22</v>
+      <c r="A39" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" t="s">
+        <v>21</v>
       </c>
       <c r="C39">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B40" s="42" t="s">
-        <v>22</v>
+      <c r="A40" t="s">
+        <v>31</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41" s="42" t="s">
-        <v>23</v>
+      <c r="A41" t="s">
+        <v>29</v>
+      </c>
+      <c r="B41" t="s">
+        <v>22</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="42" t="s">
-        <v>23</v>
+      <c r="A42" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" t="s">
+        <v>22</v>
       </c>
       <c r="C42">
         <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="B43" s="42" t="s">
-        <v>23</v>
+      <c r="A43" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" t="s">
+        <v>22</v>
       </c>
       <c r="C43">
         <v>1</v>

</xml_diff>